<commit_message>
added add to cart flow 5/8/26
</commit_message>
<xml_diff>
--- a/TestData/AddToCart.xlsx
+++ b/TestData/AddToCart.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Developer\eclipse-workspace\com.titan.eyestage\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teste\Titan-Mobile-Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C5C3B7-5403-4B17-9C70-CF0362AD0DA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24B15848-1ED5-48D7-9CDD-FA71658F4D44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6000" yWindow="4125" windowWidth="14490" windowHeight="6795" xr2:uid="{53B419D7-5DEB-49AD-9CDA-B1EC0FCC8D92}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,15 +30,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="9">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -51,17 +49,26 @@
     <t>CLSKU</t>
   </si>
   <si>
-    <t>TW1091WHM1</t>
-  </si>
-  <si>
     <t>FrameSKU</t>
+  </si>
+  <si>
+    <t>PoweredSunglassSKU</t>
+  </si>
+  <si>
+    <t>RxP222GR1 </t>
+  </si>
+  <si>
+    <t>CBUTWD85</t>
+  </si>
+  <si>
+    <t>P449BK3TIEV</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -71,9 +78,15 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="Consolas"/>
-      <family val="3"/>
+      <color rgb="FF0F1D2A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0F1D2A"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -96,9 +109,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -412,17 +426,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0575140-7AB2-45AF-BF16-5E710AC1DE63}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B1BECAA-E7C3-4729-9704-A408DC33D20C}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="2" max="2" width="22.28515625" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" customWidth="1"/>
+    <col min="5" max="5" width="17.44140625" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -435,23 +451,64 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>4</v>
-      </c>
+      <c r="C2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02CAD0B7-4C47-44E3-ACD2-2B082261F449}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Completed the payment scripts
</commit_message>
<xml_diff>
--- a/TestData/AddToCart.xlsx
+++ b/TestData/AddToCart.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Paresh automation\Titan-Mobile-Automation\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teste\Titan-Mobile-Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{156E6110-42D1-411C-BA99-31C6DC251555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8744205C-2B34-4A5C-BCFA-4ACA8272CAD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,9 +29,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -565,20 +561,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B1BECAA-E7C3-4729-9704-A408DC33D20C}">
   <dimension ref="A1:J42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
-    <col min="5" max="5" width="17.42578125" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="15.140625" customWidth="1"/>
-    <col min="8" max="8" width="23.7109375" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="17.44140625" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" customWidth="1"/>
+    <col min="9" max="9" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -610,7 +606,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -628,99 +624,99 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="I14" s="8"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="I15" s="9"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="D16" s="8"/>
       <c r="I16" s="9"/>
     </row>
-    <row r="17" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D17" s="9"/>
       <c r="I17" s="9"/>
     </row>
-    <row r="18" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D18" s="9"/>
       <c r="I18" s="9"/>
     </row>
-    <row r="19" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D19" s="10"/>
       <c r="I19" s="9"/>
     </row>
-    <row r="20" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D20" s="9"/>
       <c r="I20" s="10"/>
     </row>
-    <row r="21" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D21" s="10"/>
     </row>
-    <row r="22" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="4:9" x14ac:dyDescent="0.3">
       <c r="I22" s="9"/>
     </row>
-    <row r="23" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D23" s="8"/>
       <c r="I23" s="9"/>
     </row>
-    <row r="24" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D24" s="8"/>
       <c r="I24" s="9"/>
     </row>
-    <row r="25" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D25" s="9"/>
       <c r="I25" s="9"/>
     </row>
-    <row r="26" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D26" s="10"/>
       <c r="I26" s="9"/>
     </row>
-    <row r="27" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D27" s="9"/>
       <c r="I27" s="10"/>
     </row>
-    <row r="28" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D28" s="10"/>
     </row>
-    <row r="29" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="4:9" x14ac:dyDescent="0.3">
       <c r="I29" s="8"/>
     </row>
-    <row r="30" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="4:9" x14ac:dyDescent="0.3">
       <c r="I30" s="9"/>
     </row>
-    <row r="31" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="4:9" x14ac:dyDescent="0.3">
       <c r="G31" s="10"/>
       <c r="I31" s="9"/>
     </row>
-    <row r="32" spans="4:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="4:9" x14ac:dyDescent="0.3">
       <c r="I32" s="9"/>
     </row>
-    <row r="33" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I33" s="10"/>
     </row>
-    <row r="34" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I34" s="9"/>
     </row>
-    <row r="35" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I35" s="10"/>
     </row>
-    <row r="37" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I37" s="9"/>
     </row>
-    <row r="38" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I38" s="9"/>
     </row>
-    <row r="39" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I39" s="9"/>
     </row>
-    <row r="40" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I40" s="9"/>
     </row>
-    <row r="41" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I41" s="9"/>
     </row>
-    <row r="42" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I42" s="10"/>
     </row>
   </sheetData>
@@ -732,12 +728,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02CAD0B7-4C47-44E3-ACD2-2B082261F449}">
   <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="9" max="9" width="32.5703125" customWidth="1"/>
+    <col min="9" max="9" width="32.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -766,7 +762,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -795,12 +791,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="D3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>8</v>
       </c>
@@ -823,7 +819,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -852,7 +848,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B11" s="5" t="s">
         <v>8</v>
       </c>
@@ -875,27 +871,27 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="H14" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="H15" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="H16" s="12" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H17" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H18" s="12" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Harden v2 purchase flow against transient Appium/BrowserStack driver errors
Shared CommonUtils waits (click, visibilityOf, sendKeys, getText, etc.) now
ignore transient WebDriverException while polling instead of failing on the
first driver hiccup, so a momentary "Session not started" / "unexpected
driver response" from Appium/UIAutomator2 gets retried within the existing
30s wait budget instead of aborting the step. Added a matching retry around
the Razorpay webview context-attach in PaymentPageElements, handled the
address-selection screen in the purchase journey, cross-producted purchase
cases with every configured device in PurchaseDataProviderUtil, and dropped
purchase-suite parallelism to 1 device at a time after parallel BrowserStack
sessions proved to be the main source of this flakiness.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016eMuVRqvEfMxiYbzHGBb5C
</commit_message>
<xml_diff>
--- a/TestData/AddToCart.xlsx
+++ b/TestData/AddToCart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teste\Titan-Mobile-Automation\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Paresh automation\Titan-Mobile-Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E31C17E-A22F-4A12-933D-69E05ADA7199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9600A1D-2DF5-41A4-B9FC-E8E6F73536CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{42D689F5-8BC2-464B-8241-B0624ACD5F18}"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
@@ -31,12 +31,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="30">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -568,21 +571,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B1BECAA-E7C3-4729-9704-A408DC33D20C}">
   <dimension ref="A1:K42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" customWidth="1"/>
-    <col min="5" max="5" width="17.44140625" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" customWidth="1"/>
-    <col min="7" max="7" width="15.109375" customWidth="1"/>
-    <col min="8" max="8" width="23.6640625" customWidth="1"/>
-    <col min="9" max="9" width="20.6640625" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="17.42578125" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" customWidth="1"/>
+    <col min="8" max="8" width="23.7109375" customWidth="1"/>
+    <col min="9" max="9" width="20.7109375" customWidth="1"/>
     <col min="10" max="10" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -617,7 +620,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -631,225 +634,142 @@
       <c r="G2" s="5"/>
       <c r="H2" s="4"/>
       <c r="I2" s="6"/>
-      <c r="J2" s="12" t="s">
-        <v>27</v>
+      <c r="J2" t="s">
+        <v>22</v>
       </c>
       <c r="K2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="J3" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="K3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4" t="s">
-        <v>22</v>
-      </c>
-      <c r="K4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J5" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="K5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="K6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C3" s="5"/>
+      <c r="J3" s="12"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="11"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="12"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I14" s="8"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I15" s="9"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D16" s="8"/>
       <c r="I16" s="9"/>
     </row>
-    <row r="17" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D17" s="9"/>
       <c r="I17" s="9"/>
     </row>
-    <row r="18" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D18" s="9"/>
       <c r="I18" s="9"/>
     </row>
-    <row r="19" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D19" s="10"/>
       <c r="I19" s="9"/>
     </row>
-    <row r="20" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D20" s="9"/>
       <c r="I20" s="10"/>
     </row>
-    <row r="21" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D21" s="10"/>
     </row>
-    <row r="22" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I22" s="9"/>
     </row>
-    <row r="23" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D23" s="8"/>
       <c r="I23" s="9"/>
     </row>
-    <row r="24" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D24" s="8"/>
       <c r="I24" s="9"/>
     </row>
-    <row r="25" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D25" s="9"/>
       <c r="I25" s="9"/>
     </row>
-    <row r="26" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D26" s="10"/>
       <c r="I26" s="9"/>
     </row>
-    <row r="27" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D27" s="9"/>
       <c r="I27" s="10"/>
     </row>
-    <row r="28" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D28" s="10"/>
     </row>
-    <row r="29" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I29" s="8"/>
     </row>
-    <row r="30" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I30" s="9"/>
     </row>
-    <row r="31" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="4:9" x14ac:dyDescent="0.25">
       <c r="G31" s="10"/>
       <c r="I31" s="9"/>
     </row>
-    <row r="32" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="4:9" x14ac:dyDescent="0.25">
       <c r="I32" s="9"/>
     </row>
-    <row r="33" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I33" s="10"/>
     </row>
-    <row r="34" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I34" s="9"/>
     </row>
-    <row r="35" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I35" s="10"/>
     </row>
-    <row r="37" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I37" s="9"/>
     </row>
-    <row r="38" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I38" s="9"/>
     </row>
-    <row r="39" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I39" s="9"/>
     </row>
-    <row r="40" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I40" s="9"/>
     </row>
-    <row r="41" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I41" s="9"/>
     </row>
-    <row r="42" spans="9:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="9:9" x14ac:dyDescent="0.25">
       <c r="I42" s="10"/>
     </row>
   </sheetData>
@@ -861,12 +781,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02CAD0B7-4C47-44E3-ACD2-2B082261F449}">
   <dimension ref="A1:J51"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="9" max="9" width="32.5546875" customWidth="1"/>
+    <col min="9" max="9" width="32.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -895,7 +815,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -924,12 +844,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="D3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
         <v>8</v>
       </c>
@@ -952,7 +872,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -981,7 +901,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B11" s="5" t="s">
         <v>8</v>
       </c>
@@ -1004,32 +924,32 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H14" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H15" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H16" s="12" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H17" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H18" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>0</v>
       </c>
@@ -1061,7 +981,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>1</v>
       </c>
@@ -1079,7 +999,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2</v>
       </c>
@@ -1090,7 +1010,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>3</v>
       </c>
@@ -1122,7 +1042,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>4</v>
       </c>
@@ -1154,7 +1074,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>5</v>
       </c>
@@ -1194,9 +1114,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D340067D-92C5-4A87-863D-4C9C26FE9C40}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1228,7 +1148,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1246,7 +1166,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1257,7 +1177,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1289,7 +1209,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1321,7 +1241,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1353,7 +1273,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1367,7 +1287,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>3</v>
       </c>
@@ -1402,7 +1322,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>4</v>
       </c>
@@ -1437,7 +1357,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>5</v>
       </c>

</xml_diff>